<commit_message>
docs: registrar pruebas en Android, validación manual aprobada y nuevas evidencias
</commit_message>
<xml_diff>
--- a/docs/PRUEBAS.xlsx
+++ b/docs/PRUEBAS.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matriz de riesgos" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de prueba'!$A$1:$I$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Casos de prueba'!$A$1:$I$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Matriz de riesgos'!$A$1:$G$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -992,12 +992,12 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>1. Claves AIza…/sk-…/ambiguas</t>
+          <t>1. Claves AIza…/AQ./sk-…/ambiguas</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Detecta Gemini/OpenAI; ambiguas → null (selector manual); sk-ant- no se confunde</t>
+          <t>Detecta Gemini (AIza y AQ.); cualquier otro formato → null (selector manual)</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
@@ -1447,42 +1447,42 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>PRU-14</t>
+          <t>PRU-23</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>Ejecución en Android</t>
+          <t>Probar conexión con la clave guardada (Android)</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Teléfono Android 15 (API 35, arm64) por USB</t>
+          <t>Clave de Gemini guardada</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>1. Compilar e instalar 2. Abrir la app</t>
+          <t>1. Abrir Configuración 2. Probar conexión con el campo de clave vacío</t>
         </is>
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>App funcional</t>
+          <t>Conexión correcta usando la clave de SecureStorage</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>La primera instalación mostraba “No se pudo leer el historial local” y luego se cerraba al iniciar (paquetes SQLite mezclados 2.x/3.x). Corregido; la app corre y todas las pantallas funcionan. El emulador no es viable en este equipo (virtualización desactivada).</t>
+          <t>“Estado: Conexión correcta” y “Conexión correcta con el proveedor.”</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Aprobado (corregido)</t>
+          <t>Aprobado</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>android_01_inicio.png</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr">
@@ -1494,52 +1494,334 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
+          <t>PRU-24</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Cargar modelos desde la UI (Android)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Clave de Gemini guardada</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>1. Pulsar Cargar modelos</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Lista de modelos de chat sin modelos de imagen, audio ni tts</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>“31 modelos disponibles.” (el proveedor devuelve 60; se excluyen los no aptos para chat).</t>
+        </is>
+      </c>
+      <c r="G23" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>android_12_modelos_cargados.png</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución en dispositivo Android físico</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>PRU-25</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Proveedores disponibles (Android)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>1. Abrir el selector de proveedor</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Solo Google Gemini y Pollinations</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>El selector muestra únicamente Google Gemini y Pollinations.</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>android_13_lista_proveedores.png</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución en dispositivo Android físico</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>PRU-26</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>Categoría y búsqueda en el historial (Android)</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Clave guardada</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>1. Consultar 2. Elegir categoría Estudio 3. Guardar 4. Buscar “SQLite” 5. Buscar texto inexistente</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>El registro conserva la categoría; el filtro muestra solo coincidencias; sin coincidencias muestra “Sin resultados”</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Segunda consulta real guardada con categoría Estudio; el filtro mostró solo ese registro; el texto inexistente mostró “Sin resultados”.</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>android_14, android_15, android_16</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución en dispositivo Android físico</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>PRU-27</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>Actualizar y eliminar desde la versión final (Android)</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Registro guardado</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>1. Abrir Detalle 2. Marcar verificada y guardar 3. Eliminar con confirmación</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Cambios guardados; registro eliminado</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>“Cambios guardados.”; confirmación; el registro dejó de aparecer en el historial. El resto del historial se conservó.</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>android_17_detalle_categoria_estudio.png</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución en dispositivo Android físico</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>PRU-28</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>Validación manual en dispositivo Android</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Aplicación instalada en el dispositivo</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>1. Uso manual de la aplicación por el estudiante</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>La aplicación funciona correctamente</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Aprobada. Confirmada por el estudiante el 23/10/2026 a las 6:26 p. m.</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>Confirmación del estudiante (sin captura)</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Manual en dispositivo Android (estudiante)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>PRU-14</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución en Android</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Teléfono Android 15 (API 35, arm64) por USB</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>1. Compilar e instalar 2. Abrir la app</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>App funcional</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>La primera instalación mostraba “No se pudo leer el historial local” y luego se cerraba al iniciar (paquetes SQLite mezclados 2.x/3.x). Corregido; la app corre y todas las pantallas funcionan. El emulador no es viable en este equipo (virtualización desactivada).</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>Aprobado (corregido)</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>android_01_inicio.png</t>
+        </is>
+      </c>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Ejecución en dispositivo Android físico</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
           <t>PRU-15</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
+      <c r="B29" s="2" t="inlineStr">
         <is>
           <t>Navegación y estados de UI en Windows</t>
         </is>
       </c>
-      <c r="C23" s="2" t="inlineStr">
+      <c r="C29" s="2" t="inlineStr">
         <is>
           <t>App Windows</t>
         </is>
       </c>
-      <c r="D23" s="2" t="inlineStr">
+      <c r="D29" s="2" t="inlineStr">
         <is>
           <t>1. Recorrer Inicio, Consultar, Historial, Detalle, Configuración</t>
         </is>
       </c>
-      <c r="E23" s="2" t="inlineStr">
+      <c r="E29" s="2" t="inlineStr">
         <is>
           <t>Pantallas visibles, estados vacío/aviso correctos</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
+      <c r="F29" s="2" t="inlineStr">
         <is>
           <t>Las cinco pantallas se ejecutaron y capturaron.</t>
         </is>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Aprobado</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
+      <c r="H29" s="2" t="inlineStr">
         <is>
           <t>docs/evidencias/01–07</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr">
+      <c r="I29" s="2" t="inlineStr">
         <is>
           <t>Manual en Windows</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I23"/>
+  <autoFilter ref="A1:I29"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1575,7 +1857,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3">
@@ -1628,7 +1910,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Suite automática: 51 pruebas xUnit (5 en vivo opcionales que solo corren con variables de entorno), 0 fallos. Los tipos de ejecución están en la columna I. El detalle del dispositivo Android está en la hoja “Registro Android”.</t>
+          <t>Suite automática: 52 pruebas xUnit (5 en vivo opcionales que solo corren con variables de entorno), 0 fallos. Los tipos de ejecución están en la columna I. El detalle del dispositivo Android está en la hoja “Registro Android”.</t>
         </is>
       </c>
     </row>
@@ -1643,7 +1925,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="38" customWidth="1" min="1" max="1"/>
@@ -1682,7 +1964,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>No registrado</t>
+          <t>23129RA5FL (código del dispositivo)</t>
         </is>
       </c>
     </row>
@@ -1754,31 +2036,43 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Acciones sobre la interfaz y capturas realizadas desde el equipo de desarrollo con adb; casos PRU-14 y PRU-18 a PRU-22 (evidencias android_*.png en docs/evidencias).</t>
+          <t>Acciones sobre la interfaz y capturas realizadas desde el equipo de desarrollo con adb; casos PRU-14 y PRU-18 a PRU-27 (evidencias android_*.png en docs/evidencias). La validación manual del estudiante se registra en PRU-28.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Validación manual libre del estudiante</t>
+          <t>Validación manual en dispositivo Android</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Declarada por el estudiante (la aplicación funciona según su comprobación). Casos individuales, fecha y resultados detallados: No registrado; pendiente de confirmación.</t>
+          <t>Aprobada. El estudiante confirmó que la aplicación funciona correctamente en el dispositivo (caso PRU-28).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Alcance no verificado en Android</t>
+          <t>Fecha y hora de la validación manual</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Búsqueda en el historial, categorías distintas de General, tiempo de espera, límite 429 y proveedores distintos de Gemini: No ejecutado en el dispositivo.</t>
+          <t>23/10/2026, 6:26 p. m.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Alcance no ejecutado en Android</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Tiempo de espera agotado y límite 429 (verificados solo con pruebas automatizadas) y proveedor Pollinations con clave.</t>
         </is>
       </c>
     </row>

</xml_diff>